<commit_message>
Descarga nacional completa (rural 3.146.344 predios); pais organizado y datos del visor, estadisticas y Excel regenerados
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/datos/municipios_boyaca.xlsx
+++ b/docs/datos/municipios_boyaca.xlsx
@@ -17,7 +17,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Municipios'!$A$1:$BD$124</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Provincias'!$A$1:$J$14</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Jerarquia'!$A$1:$M$124</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Coincidencias'!$A$1:$W$124</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Coincidencias'!$A$1:$W$125</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Fuentes'!$A$1:$C$6</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -29321,7 +29321,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W124"/>
+  <dimension ref="A1:W125"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -39425,8 +39425,59 @@
         <v>1</v>
       </c>
     </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>15000</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr"/>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>Sin_Nombre_Divipola</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr"/>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>Solo en el repositorio</t>
+        </is>
+      </c>
+      <c r="F125" t="inlineStr"/>
+      <c r="G125" t="inlineStr"/>
+      <c r="H125" t="inlineStr"/>
+      <c r="I125" t="inlineStr"/>
+      <c r="J125" t="inlineStr"/>
+      <c r="K125" t="inlineStr"/>
+      <c r="L125" t="inlineStr"/>
+      <c r="M125" t="inlineStr"/>
+      <c r="N125" t="inlineStr"/>
+      <c r="O125" t="inlineStr"/>
+      <c r="P125" t="inlineStr"/>
+      <c r="Q125" t="n">
+        <v>4</v>
+      </c>
+      <c r="R125" t="n">
+        <v>1.406186</v>
+      </c>
+      <c r="S125" t="n">
+        <v>1</v>
+      </c>
+      <c r="T125" t="n">
+        <v>0.005966</v>
+      </c>
+      <c r="U125" t="n">
+        <v>3</v>
+      </c>
+      <c r="V125" t="n">
+        <v>1.157721</v>
+      </c>
+      <c r="W125" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:W124"/>
+  <autoFilter ref="A1:W125"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>